<commit_message>
antes de hacer los cambios en las materias
</commit_message>
<xml_diff>
--- a/backend/templates/notasCertificadasTest.xlsx
+++ b/backend/templates/notasCertificadasTest.xlsx
@@ -5,16 +5,40 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Axioma\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JavierWorkSpace\BatallaProject\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66B1A301-2E42-44A7-A357-E5FBBC41B4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD40A9C4-03E7-4E5F-9B1E-4E6F6C6E15C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="915" windowWidth="29040" windowHeight="15720" xr2:uid="{4829F978-A2A2-4D4E-869F-B9BEE6284F77}"/>
+    <workbookView xWindow="-28800" yWindow="1935" windowWidth="28800" windowHeight="15345" xr2:uid="{4829F978-A2A2-4D4E-869F-B9BEE6284F77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="cdcee">Sheet1!$B$10</definedName>
+    <definedName name="education_code">Sheet1!$B$3</definedName>
+    <definedName name="education_type">Sheet1!$B$4</definedName>
+    <definedName name="expedition_place_date">Sheet1!$B$5</definedName>
+    <definedName name="plantel_address">Sheet1!$B$6</definedName>
+    <definedName name="plantel_code">Sheet1!$B$1</definedName>
+    <definedName name="plantel_municipality">Sheet1!$B$7</definedName>
+    <definedName name="plantel_name">Sheet1!$B$2</definedName>
+    <definedName name="plantel_phone">Sheet1!$B$8</definedName>
+    <definedName name="plantel_state">Sheet1!$B$9</definedName>
+    <definedName name="student_birth_country">Sheet1!$B$15</definedName>
+    <definedName name="student_birth_municipality">Sheet1!$B$17</definedName>
+    <definedName name="student_birth_state">Sheet1!$B$16</definedName>
+    <definedName name="student_birthdate">Sheet1!$B$12</definedName>
+    <definedName name="student_doc">Sheet1!$B$11</definedName>
+    <definedName name="student_firstname">Sheet1!$B$14</definedName>
+    <definedName name="student_lastname">Sheet1!$B$13</definedName>
+    <definedName name="year_1_name">Sheet1!$B$19</definedName>
+    <definedName name="year_2_name">Sheet1!$B$20</definedName>
+    <definedName name="year_3_name">Sheet1!$B$21</definedName>
+    <definedName name="year_4_name">Sheet1!$B$22</definedName>
+    <definedName name="year_5_name">Sheet1!$B$23</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>plantel_code</t>
   </si>
@@ -87,6 +111,21 @@
   </si>
   <si>
     <t>student_birth_municipality</t>
+  </si>
+  <si>
+    <t>year_1_name</t>
+  </si>
+  <si>
+    <t>year_2_name</t>
+  </si>
+  <si>
+    <t>year_3_name</t>
+  </si>
+  <si>
+    <t>year_4_name</t>
+  </si>
+  <si>
+    <t>year_5_name</t>
   </si>
 </sst>
 </file>
@@ -458,10 +497,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{799C3B72-358F-4591-8712-8C3D10141F41}">
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.140625" customWidth="1"/>
+    <col min="1" max="1" width="26.5703125" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -550,7 +589,33 @@
         <v>16</v>
       </c>
     </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>